<commit_message>
Eyeblink Transition 추가 및 씬 작업
Eyeblink 트랜지션은 미사용
</commit_message>
<xml_diff>
--- a/resource/Script/script_InertiaLucis.xlsx
+++ b/resource/Script/script_InertiaLucis.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\usosctheater\resource\Script\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{120B64F0-3016-42BF-851C-B753A1CAC160}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{343E31F3-FA61-4022-9CA7-8120B913415D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="51840" windowHeight="21120" activeTab="2" xr2:uid="{12160F34-6A21-4287-85A5-86880D8D3A1A}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2313" uniqueCount="789">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2314" uniqueCount="788">
   <si>
     <t>se_trans_out|se_trans_in</t>
   </si>
@@ -2147,22 +2147,6 @@
     <phoneticPr fontId="3" type="noConversion"/>
   </si>
   <si>
-    <t>eyeblink</t>
-    <phoneticPr fontId="3" type="noConversion"/>
-  </si>
-  <si>
-    <t>TRANSITION</t>
-    <phoneticPr fontId="3" type="noConversion"/>
-  </si>
-  <si>
-    <t>fadeout</t>
-    <phoneticPr fontId="3" type="noConversion"/>
-  </si>
-  <si>
-    <t>1등 못하면 용서 안할거니까…</t>
-    <phoneticPr fontId="3" type="noConversion"/>
-  </si>
-  <si>
     <t>SNS에서 후유코쨩이 좋은 얼굴을 하고 있다고 화제가 되고 있슴다.</t>
     <phoneticPr fontId="3" type="noConversion"/>
   </si>
@@ -2670,6 +2654,18 @@
   </si>
   <si>
     <t>smile1 face_close3 lip_smile</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>… 1등 못하면 용서 안할거니까…</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>se_taoreru</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>0.4</t>
     <phoneticPr fontId="3" type="noConversion"/>
   </si>
 </sst>
@@ -2720,7 +2716,7 @@
       <charset val="129"/>
     </font>
   </fonts>
-  <fills count="6">
+  <fills count="5">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -2736,12 +2732,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="1"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFF0000"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -2792,7 +2782,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -2818,9 +2808,6 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1">
       <alignment vertical="center"/>
     </xf>
   </cellXfs>
@@ -3302,7 +3289,7 @@
     </row>
     <row r="3" spans="2:16" x14ac:dyDescent="0.3">
       <c r="B3" s="1" t="s">
-        <v>783</v>
+        <v>779</v>
       </c>
       <c r="C3" s="1"/>
       <c r="D3" s="1"/>
@@ -3312,7 +3299,7 @@
       <c r="H3" s="1"/>
       <c r="I3" s="1"/>
       <c r="J3" s="1" t="s">
-        <v>785</v>
+        <v>781</v>
       </c>
       <c r="K3" s="1"/>
       <c r="L3" s="1"/>
@@ -4170,7 +4157,7 @@
     </row>
     <row r="33" spans="2:16" x14ac:dyDescent="0.3">
       <c r="B33" s="1" t="s">
-        <v>783</v>
+        <v>779</v>
       </c>
       <c r="C33" s="1"/>
       <c r="D33" s="1"/>
@@ -4180,7 +4167,7 @@
       <c r="H33" s="1"/>
       <c r="I33" s="1"/>
       <c r="J33" s="1" t="s">
-        <v>785</v>
+        <v>781</v>
       </c>
       <c r="K33" s="1"/>
       <c r="L33" s="1"/>
@@ -5355,7 +5342,7 @@
     </row>
     <row r="76" spans="2:16" x14ac:dyDescent="0.3">
       <c r="B76" s="1" t="s">
-        <v>784</v>
+        <v>780</v>
       </c>
       <c r="C76" s="1"/>
       <c r="D76" s="1"/>
@@ -5365,7 +5352,7 @@
       <c r="H76" s="1"/>
       <c r="I76" s="1"/>
       <c r="J76" s="1" t="s">
-        <v>785</v>
+        <v>781</v>
       </c>
       <c r="K76" s="1"/>
       <c r="L76" s="1"/>
@@ -6493,7 +6480,7 @@
     </row>
     <row r="3" spans="2:16" x14ac:dyDescent="0.3">
       <c r="B3" s="1" t="s">
-        <v>783</v>
+        <v>779</v>
       </c>
       <c r="C3" s="1"/>
       <c r="D3" s="1"/>
@@ -6503,7 +6490,7 @@
       <c r="H3" s="1"/>
       <c r="I3" s="1"/>
       <c r="J3" s="1" t="s">
-        <v>785</v>
+        <v>781</v>
       </c>
       <c r="K3" s="1"/>
       <c r="L3" s="1"/>
@@ -11139,7 +11126,7 @@
     </row>
     <row r="4" spans="2:16" x14ac:dyDescent="0.3">
       <c r="B4" s="1" t="s">
-        <v>783</v>
+        <v>779</v>
       </c>
       <c r="C4" s="1"/>
       <c r="D4" s="1"/>
@@ -11149,12 +11136,12 @@
       <c r="H4" s="1"/>
       <c r="I4" s="1"/>
       <c r="J4" s="1" t="s">
-        <v>785</v>
+        <v>781</v>
       </c>
       <c r="K4" s="1"/>
       <c r="L4" s="1"/>
       <c r="M4" s="1" t="s">
-        <v>771</v>
+        <v>767</v>
       </c>
       <c r="N4" s="1" t="s">
         <v>106</v>
@@ -11194,7 +11181,7 @@
         <v>548</v>
       </c>
       <c r="E6" s="1" t="s">
-        <v>677</v>
+        <v>673</v>
       </c>
       <c r="F6" s="1" t="s">
         <v>293</v>
@@ -11227,7 +11214,7 @@
         <v>549</v>
       </c>
       <c r="E7" s="1" t="s">
-        <v>679</v>
+        <v>675</v>
       </c>
       <c r="F7" s="1" t="s">
         <v>556</v>
@@ -11236,7 +11223,7 @@
         <v>121</v>
       </c>
       <c r="H7" s="1" t="s">
-        <v>778</v>
+        <v>774</v>
       </c>
       <c r="I7" s="1"/>
       <c r="J7" s="1"/>
@@ -11260,7 +11247,7 @@
         <v>550</v>
       </c>
       <c r="E8" s="1" t="s">
-        <v>678</v>
+        <v>674</v>
       </c>
       <c r="F8" s="1" t="s">
         <v>293</v>
@@ -11293,7 +11280,7 @@
         <v>553</v>
       </c>
       <c r="E9" s="1" t="s">
-        <v>680</v>
+        <v>676</v>
       </c>
       <c r="F9" s="1" t="s">
         <v>52</v>
@@ -11343,7 +11330,7 @@
         <v>554</v>
       </c>
       <c r="E11" s="1" t="s">
-        <v>681</v>
+        <v>677</v>
       </c>
       <c r="F11" s="1" t="s">
         <v>556</v>
@@ -11352,7 +11339,7 @@
         <v>121</v>
       </c>
       <c r="H11" s="1" t="s">
-        <v>779</v>
+        <v>775</v>
       </c>
       <c r="I11" s="1"/>
       <c r="J11" s="1"/>
@@ -11376,7 +11363,7 @@
         <v>555</v>
       </c>
       <c r="E12" s="1" t="s">
-        <v>682</v>
+        <v>678</v>
       </c>
       <c r="F12" s="1" t="s">
         <v>293</v>
@@ -11385,7 +11372,7 @@
         <v>12</v>
       </c>
       <c r="H12" s="1" t="s">
-        <v>776</v>
+        <v>772</v>
       </c>
       <c r="I12" s="1"/>
       <c r="J12" s="1"/>
@@ -11409,7 +11396,7 @@
         <v>559</v>
       </c>
       <c r="E13" s="1" t="s">
-        <v>683</v>
+        <v>679</v>
       </c>
       <c r="F13" s="1" t="s">
         <v>557</v>
@@ -11442,7 +11429,7 @@
         <v>560</v>
       </c>
       <c r="E14" s="1" t="s">
-        <v>684</v>
+        <v>680</v>
       </c>
       <c r="F14" s="1"/>
       <c r="G14" s="1"/>
@@ -11468,7 +11455,7 @@
         <v>561</v>
       </c>
       <c r="E15" s="1" t="s">
-        <v>685</v>
+        <v>681</v>
       </c>
       <c r="F15" s="1" t="s">
         <v>293</v>
@@ -11501,7 +11488,7 @@
         <v>563</v>
       </c>
       <c r="E16" s="1" t="s">
-        <v>686</v>
+        <v>682</v>
       </c>
       <c r="F16" s="1" t="s">
         <v>293</v>
@@ -11510,7 +11497,7 @@
         <v>12</v>
       </c>
       <c r="H16" s="1" t="s">
-        <v>770</v>
+        <v>766</v>
       </c>
       <c r="I16" s="1"/>
       <c r="J16" s="1"/>
@@ -11534,7 +11521,7 @@
         <v>564</v>
       </c>
       <c r="E17" s="1" t="s">
-        <v>687</v>
+        <v>683</v>
       </c>
       <c r="F17" s="1"/>
       <c r="G17" s="1"/>
@@ -11561,7 +11548,7 @@
         <v>565</v>
       </c>
       <c r="E18" s="1" t="s">
-        <v>688</v>
+        <v>684</v>
       </c>
       <c r="F18" s="1" t="s">
         <v>557</v>
@@ -11594,7 +11581,7 @@
         <v>567</v>
       </c>
       <c r="E19" s="1" t="s">
-        <v>689</v>
+        <v>685</v>
       </c>
       <c r="F19" s="1" t="s">
         <v>293</v>
@@ -11696,7 +11683,7 @@
         <v>569</v>
       </c>
       <c r="E23" s="1" t="s">
-        <v>690</v>
+        <v>686</v>
       </c>
       <c r="F23" s="1" t="s">
         <v>293</v>
@@ -11729,7 +11716,7 @@
         <v>571</v>
       </c>
       <c r="E24" s="1" t="s">
-        <v>692</v>
+        <v>688</v>
       </c>
       <c r="F24" s="1"/>
       <c r="G24" s="1"/>
@@ -11756,7 +11743,7 @@
         <v>572</v>
       </c>
       <c r="E25" s="1" t="s">
-        <v>693</v>
+        <v>689</v>
       </c>
       <c r="F25" s="1" t="s">
         <v>293</v>
@@ -11789,7 +11776,7 @@
         <v>573</v>
       </c>
       <c r="E26" s="1" t="s">
-        <v>694</v>
+        <v>690</v>
       </c>
       <c r="F26" s="1" t="s">
         <v>557</v>
@@ -11798,7 +11785,7 @@
         <v>5</v>
       </c>
       <c r="H26" t="s">
-        <v>777</v>
+        <v>773</v>
       </c>
       <c r="I26" s="1"/>
       <c r="J26" s="1"/>
@@ -11822,7 +11809,7 @@
         <v>574</v>
       </c>
       <c r="E27" s="1" t="s">
-        <v>695</v>
+        <v>691</v>
       </c>
       <c r="F27" s="1" t="s">
         <v>293</v>
@@ -11960,7 +11947,7 @@
         <v>575</v>
       </c>
       <c r="E33" s="1" t="s">
-        <v>696</v>
+        <v>692</v>
       </c>
       <c r="F33" s="1"/>
       <c r="G33" s="1"/>
@@ -11987,7 +11974,7 @@
         <v>576</v>
       </c>
       <c r="E34" s="1" t="s">
-        <v>698</v>
+        <v>694</v>
       </c>
       <c r="F34" s="1"/>
       <c r="G34" s="1"/>
@@ -12014,7 +12001,7 @@
         <v>577</v>
       </c>
       <c r="E35" s="1" t="s">
-        <v>699</v>
+        <v>695</v>
       </c>
       <c r="F35" s="1"/>
       <c r="G35" s="1"/>
@@ -12071,12 +12058,12 @@
       <c r="N37" s="1"/>
       <c r="O37" s="1"/>
       <c r="P37" s="1" t="s">
-        <v>672</v>
+        <v>668</v>
       </c>
     </row>
     <row r="38" spans="2:16" x14ac:dyDescent="0.3">
       <c r="B38" s="1" t="s">
-        <v>783</v>
+        <v>779</v>
       </c>
       <c r="C38" s="1"/>
       <c r="D38" s="1"/>
@@ -12086,12 +12073,12 @@
       <c r="H38" s="1"/>
       <c r="I38" s="1"/>
       <c r="J38" s="1" t="s">
-        <v>785</v>
+        <v>781</v>
       </c>
       <c r="K38" s="1"/>
       <c r="L38" s="1"/>
       <c r="M38" s="1" t="s">
-        <v>772</v>
+        <v>768</v>
       </c>
       <c r="N38" s="1" t="s">
         <v>106</v>
@@ -12101,7 +12088,7 @@
     </row>
     <row r="39" spans="2:16" x14ac:dyDescent="0.3">
       <c r="B39" s="1" t="s">
-        <v>783</v>
+        <v>779</v>
       </c>
       <c r="C39" s="1"/>
       <c r="D39" s="1"/>
@@ -12110,7 +12097,7 @@
       <c r="G39" s="1"/>
       <c r="H39" s="1"/>
       <c r="I39" s="1" t="s">
-        <v>675</v>
+        <v>671</v>
       </c>
       <c r="J39" s="1" t="s">
         <v>608</v>
@@ -12118,7 +12105,7 @@
       <c r="K39" s="1"/>
       <c r="L39" s="1"/>
       <c r="M39" s="1" t="s">
-        <v>674</v>
+        <v>670</v>
       </c>
       <c r="N39" s="1" t="s">
         <v>106</v>
@@ -12158,7 +12145,7 @@
         <v>579</v>
       </c>
       <c r="E41" s="1" t="s">
-        <v>700</v>
+        <v>696</v>
       </c>
       <c r="F41" s="1"/>
       <c r="G41" s="1"/>
@@ -12219,7 +12206,7 @@
       <c r="N43" s="1"/>
       <c r="O43" s="1"/>
       <c r="P43" s="1" t="s">
-        <v>672</v>
+        <v>668</v>
       </c>
     </row>
     <row r="44" spans="2:16" x14ac:dyDescent="0.3">
@@ -12233,7 +12220,7 @@
         <v>580</v>
       </c>
       <c r="E44" s="1" t="s">
-        <v>701</v>
+        <v>697</v>
       </c>
       <c r="F44" s="1"/>
       <c r="G44" s="1"/>
@@ -12260,7 +12247,7 @@
         <v>582</v>
       </c>
       <c r="E45" s="1" t="s">
-        <v>702</v>
+        <v>698</v>
       </c>
       <c r="F45" s="1"/>
       <c r="G45" s="1"/>
@@ -12287,7 +12274,7 @@
         <v>583</v>
       </c>
       <c r="E46" s="1" t="s">
-        <v>703</v>
+        <v>699</v>
       </c>
       <c r="F46" s="1"/>
       <c r="G46" s="1"/>
@@ -12314,7 +12301,7 @@
         <v>584</v>
       </c>
       <c r="E47" s="1" t="s">
-        <v>704</v>
+        <v>700</v>
       </c>
       <c r="F47" s="1"/>
       <c r="G47" s="1"/>
@@ -12341,7 +12328,7 @@
         <v>585</v>
       </c>
       <c r="E48" s="1" t="s">
-        <v>705</v>
+        <v>701</v>
       </c>
       <c r="F48" s="1"/>
       <c r="G48" s="1"/>
@@ -12368,7 +12355,7 @@
         <v>586</v>
       </c>
       <c r="E49" s="1" t="s">
-        <v>706</v>
+        <v>702</v>
       </c>
       <c r="F49" s="1"/>
       <c r="G49" s="1"/>
@@ -12395,7 +12382,7 @@
         <v>587</v>
       </c>
       <c r="E50" s="1" t="s">
-        <v>707</v>
+        <v>703</v>
       </c>
       <c r="F50" s="1"/>
       <c r="G50" s="1"/>
@@ -12422,7 +12409,7 @@
         <v>588</v>
       </c>
       <c r="E51" s="1" t="s">
-        <v>708</v>
+        <v>704</v>
       </c>
       <c r="F51" s="1"/>
       <c r="G51" s="1"/>
@@ -12449,7 +12436,7 @@
         <v>589</v>
       </c>
       <c r="E52" s="1" t="s">
-        <v>709</v>
+        <v>705</v>
       </c>
       <c r="F52" s="1"/>
       <c r="G52" s="1"/>
@@ -12476,7 +12463,7 @@
         <v>590</v>
       </c>
       <c r="E53" s="1" t="s">
-        <v>710</v>
+        <v>706</v>
       </c>
       <c r="F53" s="1"/>
       <c r="G53" s="1"/>
@@ -12529,7 +12516,7 @@
       <c r="N55" s="1"/>
       <c r="O55" s="1"/>
       <c r="P55" s="1" t="s">
-        <v>671</v>
+        <v>667</v>
       </c>
     </row>
     <row r="56" spans="2:16" x14ac:dyDescent="0.3">
@@ -12561,10 +12548,10 @@
         <v>16</v>
       </c>
       <c r="D57" s="1" t="s">
-        <v>774</v>
+        <v>770</v>
       </c>
       <c r="E57" s="1" t="s">
-        <v>711</v>
+        <v>707</v>
       </c>
       <c r="F57" s="1" t="s">
         <v>293</v>
@@ -12591,13 +12578,13 @@
         <v>10</v>
       </c>
       <c r="C58" s="1" t="s">
-        <v>775</v>
+        <v>771</v>
       </c>
       <c r="D58" s="1" t="s">
         <v>592</v>
       </c>
       <c r="E58" s="1" t="s">
-        <v>691</v>
+        <v>687</v>
       </c>
       <c r="F58" s="1" t="s">
         <v>52</v>
@@ -12620,13 +12607,13 @@
         <v>10</v>
       </c>
       <c r="C59" s="1" t="s">
-        <v>775</v>
+        <v>771</v>
       </c>
       <c r="D59" s="1" t="s">
         <v>593</v>
       </c>
       <c r="E59" s="1" t="s">
-        <v>712</v>
+        <v>708</v>
       </c>
       <c r="F59" s="1"/>
       <c r="G59" s="1"/>
@@ -12653,7 +12640,7 @@
         <v>594</v>
       </c>
       <c r="E60" s="1" t="s">
-        <v>713</v>
+        <v>709</v>
       </c>
       <c r="F60" s="1" t="s">
         <v>293</v>
@@ -12686,7 +12673,7 @@
         <v>596</v>
       </c>
       <c r="E61" s="1" t="s">
-        <v>714</v>
+        <v>710</v>
       </c>
       <c r="F61" s="1" t="s">
         <v>52</v>
@@ -12715,7 +12702,7 @@
         <v>597</v>
       </c>
       <c r="E62" s="1" t="s">
-        <v>715</v>
+        <v>711</v>
       </c>
       <c r="F62" s="1"/>
       <c r="G62" s="1"/>
@@ -12742,7 +12729,7 @@
         <v>598</v>
       </c>
       <c r="E63" s="1" t="s">
-        <v>697</v>
+        <v>693</v>
       </c>
       <c r="F63" s="1" t="s">
         <v>293</v>
@@ -12787,7 +12774,7 @@
     </row>
     <row r="65" spans="2:16" x14ac:dyDescent="0.3">
       <c r="B65" s="1" t="s">
-        <v>783</v>
+        <v>779</v>
       </c>
       <c r="C65" s="1"/>
       <c r="D65" s="1"/>
@@ -12796,10 +12783,10 @@
       <c r="G65" s="1"/>
       <c r="H65" s="1"/>
       <c r="I65" s="1" t="s">
-        <v>786</v>
+        <v>782</v>
       </c>
       <c r="J65" s="1" t="s">
-        <v>785</v>
+        <v>781</v>
       </c>
       <c r="K65" s="1"/>
       <c r="L65" s="1"/>
@@ -12810,7 +12797,7 @@
     </row>
     <row r="66" spans="2:16" x14ac:dyDescent="0.3">
       <c r="B66" s="1" t="s">
-        <v>783</v>
+        <v>779</v>
       </c>
       <c r="C66" s="1"/>
       <c r="D66" s="1"/>
@@ -12819,7 +12806,7 @@
       <c r="G66" s="1"/>
       <c r="H66" s="1"/>
       <c r="I66" s="1" t="s">
-        <v>786</v>
+        <v>782</v>
       </c>
       <c r="J66" s="1" t="s">
         <v>608</v>
@@ -13223,7 +13210,7 @@
     </row>
     <row r="83" spans="1:16" x14ac:dyDescent="0.3">
       <c r="B83" s="1" t="s">
-        <v>673</v>
+        <v>669</v>
       </c>
       <c r="C83" s="1"/>
       <c r="D83" s="1"/>
@@ -13239,13 +13226,13 @@
       <c r="N83" s="1"/>
       <c r="O83" s="1"/>
       <c r="P83" s="1" t="s">
-        <v>672</v>
+        <v>668</v>
       </c>
     </row>
     <row r="84" spans="1:16" x14ac:dyDescent="0.3">
-      <c r="A84" s="9"/>
+      <c r="A84" s="8"/>
       <c r="B84" s="1" t="s">
-        <v>783</v>
+        <v>779</v>
       </c>
       <c r="C84" s="1"/>
       <c r="D84" s="1"/>
@@ -13255,12 +13242,12 @@
       <c r="H84" s="1"/>
       <c r="I84" s="1"/>
       <c r="J84" s="1" t="s">
-        <v>785</v>
+        <v>781</v>
       </c>
       <c r="K84" s="1"/>
       <c r="L84" s="1"/>
       <c r="M84" s="1" t="s">
-        <v>773</v>
+        <v>769</v>
       </c>
       <c r="N84" s="1" t="s">
         <v>106</v>
@@ -13300,7 +13287,7 @@
         <v>601</v>
       </c>
       <c r="E86" s="1" t="s">
-        <v>716</v>
+        <v>712</v>
       </c>
       <c r="F86" s="1"/>
       <c r="G86" s="1"/>
@@ -13327,7 +13314,7 @@
         <v>602</v>
       </c>
       <c r="E87" s="1" t="s">
-        <v>717</v>
+        <v>713</v>
       </c>
       <c r="F87" s="1" t="s">
         <v>293</v>
@@ -13410,7 +13397,7 @@
         <v>604</v>
       </c>
       <c r="E90" s="1" t="s">
-        <v>769</v>
+        <v>765</v>
       </c>
       <c r="F90" s="1" t="s">
         <v>52</v>
@@ -13459,7 +13446,7 @@
         <v>605</v>
       </c>
       <c r="E92" s="1" t="s">
-        <v>718</v>
+        <v>714</v>
       </c>
       <c r="F92" s="1" t="s">
         <v>293</v>
@@ -13468,7 +13455,7 @@
         <v>20</v>
       </c>
       <c r="H92" t="s">
-        <v>781</v>
+        <v>777</v>
       </c>
       <c r="I92" s="1"/>
       <c r="J92" s="1"/>
@@ -13513,7 +13500,7 @@
         <v>606</v>
       </c>
       <c r="E94" s="1" t="s">
-        <v>719</v>
+        <v>715</v>
       </c>
       <c r="F94" s="1" t="s">
         <v>293</v>
@@ -13522,7 +13509,7 @@
         <v>20</v>
       </c>
       <c r="H94" t="s">
-        <v>788</v>
+        <v>784</v>
       </c>
       <c r="I94" s="1"/>
       <c r="J94" s="1"/>
@@ -13557,7 +13544,7 @@
       <c r="P95" s="1"/>
     </row>
     <row r="96" spans="1:16" x14ac:dyDescent="0.3">
-      <c r="A96" s="9"/>
+      <c r="A96" s="8"/>
       <c r="B96" s="1" t="s">
         <v>607</v>
       </c>
@@ -13577,7 +13564,7 @@
       </c>
       <c r="O96" s="1"/>
       <c r="P96" s="1" t="s">
-        <v>676</v>
+        <v>672</v>
       </c>
     </row>
     <row r="97" spans="2:16" x14ac:dyDescent="0.3">
@@ -13619,12 +13606,12 @@
       <c r="N98" s="1"/>
       <c r="O98" s="1"/>
       <c r="P98" s="1" t="s">
-        <v>671</v>
+        <v>667</v>
       </c>
     </row>
     <row r="99" spans="2:16" x14ac:dyDescent="0.3">
       <c r="B99" s="1" t="s">
-        <v>783</v>
+        <v>779</v>
       </c>
       <c r="C99" s="1"/>
       <c r="D99" s="1"/>
@@ -13633,7 +13620,7 @@
       <c r="G99" s="1"/>
       <c r="H99" s="1"/>
       <c r="I99" s="1" t="s">
-        <v>675</v>
+        <v>671</v>
       </c>
       <c r="J99" s="1" t="s">
         <v>608</v>
@@ -13641,7 +13628,7 @@
       <c r="K99" s="1"/>
       <c r="L99" s="1"/>
       <c r="M99" s="1" t="s">
-        <v>674</v>
+        <v>670</v>
       </c>
       <c r="N99" s="1" t="s">
         <v>106</v>
@@ -13681,7 +13668,7 @@
         <v>609</v>
       </c>
       <c r="E101" s="1" t="s">
-        <v>720</v>
+        <v>716</v>
       </c>
       <c r="F101" s="1"/>
       <c r="G101" s="1"/>
@@ -13708,7 +13695,7 @@
         <v>610</v>
       </c>
       <c r="E102" s="1" t="s">
-        <v>721</v>
+        <v>717</v>
       </c>
       <c r="F102" s="1"/>
       <c r="G102" s="1"/>
@@ -13735,7 +13722,7 @@
         <v>611</v>
       </c>
       <c r="E103" s="1" t="s">
-        <v>722</v>
+        <v>718</v>
       </c>
       <c r="F103" s="1"/>
       <c r="G103" s="1"/>
@@ -13762,7 +13749,7 @@
         <v>612</v>
       </c>
       <c r="E104" s="1" t="s">
-        <v>723</v>
+        <v>719</v>
       </c>
       <c r="F104" s="1"/>
       <c r="G104" s="1"/>
@@ -13789,7 +13776,7 @@
         <v>613</v>
       </c>
       <c r="E105" s="1" t="s">
-        <v>724</v>
+        <v>720</v>
       </c>
       <c r="F105" s="1"/>
       <c r="G105" s="1"/>
@@ -13816,7 +13803,7 @@
         <v>385</v>
       </c>
       <c r="E106" s="1" t="s">
-        <v>725</v>
+        <v>721</v>
       </c>
       <c r="I106" s="1"/>
       <c r="J106" s="1"/>
@@ -13840,7 +13827,7 @@
         <v>615</v>
       </c>
       <c r="E107" s="1" t="s">
-        <v>726</v>
+        <v>722</v>
       </c>
       <c r="F107" s="1" t="s">
         <v>293</v>
@@ -13873,7 +13860,7 @@
         <v>616</v>
       </c>
       <c r="E108" s="1" t="s">
-        <v>728</v>
+        <v>724</v>
       </c>
       <c r="F108" s="1"/>
       <c r="G108" s="1"/>
@@ -13900,7 +13887,7 @@
         <v>617</v>
       </c>
       <c r="E109" s="1" t="s">
-        <v>727</v>
+        <v>723</v>
       </c>
       <c r="F109" s="1"/>
       <c r="G109" s="1"/>
@@ -13927,7 +13914,7 @@
         <v>618</v>
       </c>
       <c r="E110" s="1" t="s">
-        <v>729</v>
+        <v>725</v>
       </c>
       <c r="F110" s="1" t="s">
         <v>52</v>
@@ -13956,7 +13943,7 @@
         <v>621</v>
       </c>
       <c r="E111" s="1" t="s">
-        <v>730</v>
+        <v>726</v>
       </c>
       <c r="F111" s="1"/>
       <c r="G111" s="1"/>
@@ -13983,7 +13970,7 @@
         <v>622</v>
       </c>
       <c r="E112" s="1" t="s">
-        <v>731</v>
+        <v>727</v>
       </c>
       <c r="F112" s="1"/>
       <c r="G112" s="1"/>
@@ -13999,7 +13986,7 @@
       <c r="O112" s="1"/>
       <c r="P112" s="1"/>
     </row>
-    <row r="113" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="113" spans="2:16" x14ac:dyDescent="0.3">
       <c r="B113" s="1" t="s">
         <v>10</v>
       </c>
@@ -14010,7 +13997,7 @@
         <v>623</v>
       </c>
       <c r="E113" s="1" t="s">
-        <v>732</v>
+        <v>728</v>
       </c>
       <c r="F113" s="1"/>
       <c r="G113" s="1"/>
@@ -14026,7 +14013,7 @@
       <c r="O113" s="1"/>
       <c r="P113" s="1"/>
     </row>
-    <row r="114" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="114" spans="2:16" x14ac:dyDescent="0.3">
       <c r="B114" s="1" t="s">
         <v>10</v>
       </c>
@@ -14037,7 +14024,7 @@
         <v>624</v>
       </c>
       <c r="E114" s="1" t="s">
-        <v>733</v>
+        <v>729</v>
       </c>
       <c r="F114" s="1"/>
       <c r="G114" s="1"/>
@@ -14053,7 +14040,7 @@
       <c r="O114" s="1"/>
       <c r="P114" s="1"/>
     </row>
-    <row r="115" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="115" spans="2:16" x14ac:dyDescent="0.3">
       <c r="B115" s="1" t="s">
         <v>10</v>
       </c>
@@ -14064,7 +14051,7 @@
         <v>625</v>
       </c>
       <c r="E115" s="1" t="s">
-        <v>734</v>
+        <v>730</v>
       </c>
       <c r="F115" s="1"/>
       <c r="G115" s="1"/>
@@ -14080,7 +14067,7 @@
       <c r="O115" s="1"/>
       <c r="P115" s="1"/>
     </row>
-    <row r="116" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="116" spans="2:16" x14ac:dyDescent="0.3">
       <c r="B116" s="1" t="s">
         <v>10</v>
       </c>
@@ -14091,7 +14078,7 @@
         <v>385</v>
       </c>
       <c r="E116" s="1" t="s">
-        <v>735</v>
+        <v>731</v>
       </c>
       <c r="F116" s="1"/>
       <c r="G116" s="1"/>
@@ -14106,7 +14093,7 @@
       <c r="O116" s="1"/>
       <c r="P116" s="1"/>
     </row>
-    <row r="117" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="117" spans="2:16" x14ac:dyDescent="0.3">
       <c r="B117" s="1" t="s">
         <v>10</v>
       </c>
@@ -14117,7 +14104,7 @@
         <v>627</v>
       </c>
       <c r="E117" s="1" t="s">
-        <v>736</v>
+        <v>732</v>
       </c>
       <c r="F117" s="1"/>
       <c r="G117" s="1"/>
@@ -14133,7 +14120,7 @@
       <c r="O117" s="1"/>
       <c r="P117" s="1"/>
     </row>
-    <row r="118" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="118" spans="2:16" x14ac:dyDescent="0.3">
       <c r="B118" s="1" t="s">
         <v>10</v>
       </c>
@@ -14144,7 +14131,7 @@
         <v>628</v>
       </c>
       <c r="E118" s="1" t="s">
-        <v>737</v>
+        <v>733</v>
       </c>
       <c r="F118" s="1"/>
       <c r="G118" s="1"/>
@@ -14160,7 +14147,7 @@
       <c r="O118" s="1"/>
       <c r="P118" s="1"/>
     </row>
-    <row r="119" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="119" spans="2:16" x14ac:dyDescent="0.3">
       <c r="B119" s="1" t="s">
         <v>10</v>
       </c>
@@ -14171,7 +14158,7 @@
         <v>629</v>
       </c>
       <c r="E119" s="1" t="s">
-        <v>738</v>
+        <v>734</v>
       </c>
       <c r="F119" s="1" t="s">
         <v>293</v>
@@ -14193,7 +14180,7 @@
       <c r="O119" s="1"/>
       <c r="P119" s="1"/>
     </row>
-    <row r="120" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="120" spans="2:16" x14ac:dyDescent="0.3">
       <c r="B120" s="1" t="s">
         <v>10</v>
       </c>
@@ -14204,7 +14191,7 @@
         <v>631</v>
       </c>
       <c r="E120" s="1" t="s">
-        <v>739</v>
+        <v>735</v>
       </c>
       <c r="F120" s="1"/>
       <c r="G120" s="1"/>
@@ -14219,7 +14206,7 @@
       <c r="O120" s="1"/>
       <c r="P120" s="1"/>
     </row>
-    <row r="121" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="121" spans="2:16" x14ac:dyDescent="0.3">
       <c r="B121" s="1" t="s">
         <v>10</v>
       </c>
@@ -14230,7 +14217,7 @@
         <v>632</v>
       </c>
       <c r="E121" s="1" t="s">
-        <v>740</v>
+        <v>736</v>
       </c>
       <c r="F121" s="1" t="s">
         <v>52</v>
@@ -14248,7 +14235,7 @@
       <c r="O121" s="1"/>
       <c r="P121" s="1"/>
     </row>
-    <row r="122" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="122" spans="2:16" x14ac:dyDescent="0.3">
       <c r="B122" s="1" t="s">
         <v>10</v>
       </c>
@@ -14259,7 +14246,7 @@
         <v>633</v>
       </c>
       <c r="E122" s="1" t="s">
-        <v>741</v>
+        <v>737</v>
       </c>
       <c r="F122" s="1" t="s">
         <v>556</v>
@@ -14268,7 +14255,7 @@
         <v>20</v>
       </c>
       <c r="H122" s="1" t="s">
-        <v>780</v>
+        <v>776</v>
       </c>
       <c r="I122" s="1"/>
       <c r="J122" s="1"/>
@@ -14281,7 +14268,7 @@
       <c r="O122" s="1"/>
       <c r="P122" s="1"/>
     </row>
-    <row r="123" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="123" spans="2:16" x14ac:dyDescent="0.3">
       <c r="B123" s="1" t="s">
         <v>2</v>
       </c>
@@ -14302,7 +14289,7 @@
       <c r="O123" s="1"/>
       <c r="P123" s="1"/>
     </row>
-    <row r="124" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="124" spans="2:16" x14ac:dyDescent="0.3">
       <c r="B124" s="1" t="s">
         <v>59</v>
       </c>
@@ -14316,14 +14303,18 @@
       <c r="J124" s="1"/>
       <c r="K124" s="1"/>
       <c r="L124" s="1"/>
-      <c r="M124" s="1"/>
-      <c r="N124" s="1"/>
+      <c r="M124" s="1" t="s">
+        <v>786</v>
+      </c>
+      <c r="N124" s="1" t="s">
+        <v>787</v>
+      </c>
       <c r="O124" s="1"/>
       <c r="P124" s="1" t="s">
-        <v>671</v>
-      </c>
-    </row>
-    <row r="125" spans="1:16" x14ac:dyDescent="0.3">
+        <v>667</v>
+      </c>
+    </row>
+    <row r="125" spans="2:16" x14ac:dyDescent="0.3">
       <c r="B125" s="1" t="s">
         <v>546</v>
       </c>
@@ -14344,7 +14335,7 @@
       <c r="O125" s="1"/>
       <c r="P125" s="1"/>
     </row>
-    <row r="126" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="126" spans="2:16" x14ac:dyDescent="0.3">
       <c r="B126" s="1" t="s">
         <v>10</v>
       </c>
@@ -14355,7 +14346,7 @@
         <v>614</v>
       </c>
       <c r="E126" s="1" t="s">
-        <v>742</v>
+        <v>738</v>
       </c>
       <c r="F126" s="1"/>
       <c r="G126" s="1"/>
@@ -14370,7 +14361,7 @@
       <c r="O126" s="1"/>
       <c r="P126" s="1"/>
     </row>
-    <row r="127" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="127" spans="2:16" x14ac:dyDescent="0.3">
       <c r="B127" s="1" t="s">
         <v>10</v>
       </c>
@@ -14381,7 +14372,7 @@
         <v>637</v>
       </c>
       <c r="E127" s="1" t="s">
-        <v>743</v>
+        <v>739</v>
       </c>
       <c r="F127" s="1"/>
       <c r="G127" s="1"/>
@@ -14396,8 +14387,7 @@
       <c r="O127" s="1"/>
       <c r="P127" s="1"/>
     </row>
-    <row r="128" spans="1:16" x14ac:dyDescent="0.3">
-      <c r="A128" s="8"/>
+    <row r="128" spans="2:16" x14ac:dyDescent="0.3">
       <c r="B128" s="1" t="s">
         <v>607</v>
       </c>
@@ -14406,10 +14396,7 @@
       <c r="E128" s="1"/>
       <c r="F128" s="1"/>
       <c r="G128" s="1"/>
-      <c r="H128" s="1"/>
-      <c r="I128" s="1" t="s">
-        <v>638</v>
-      </c>
+      <c r="I128" s="1"/>
       <c r="J128" s="1"/>
       <c r="K128" s="1"/>
       <c r="L128" s="1"/>
@@ -14418,9 +14405,9 @@
       <c r="O128" s="1"/>
       <c r="P128" s="1"/>
     </row>
-    <row r="129" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="129" spans="2:16" x14ac:dyDescent="0.3">
       <c r="B129" s="1" t="s">
-        <v>546</v>
+        <v>2</v>
       </c>
       <c r="C129" s="1"/>
       <c r="D129" s="1"/>
@@ -14429,7 +14416,7 @@
       <c r="G129" s="1"/>
       <c r="H129" s="1"/>
       <c r="I129" s="1" t="s">
-        <v>544</v>
+        <v>599</v>
       </c>
       <c r="J129" s="1"/>
       <c r="K129" s="1"/>
@@ -14439,18 +14426,18 @@
       <c r="O129" s="1"/>
       <c r="P129" s="1"/>
     </row>
-    <row r="130" spans="1:16" x14ac:dyDescent="0.3">
-      <c r="A130" s="8"/>
+    <row r="130" spans="2:16" x14ac:dyDescent="0.3">
       <c r="B130" s="1" t="s">
-        <v>639</v>
+        <v>546</v>
       </c>
       <c r="C130" s="1"/>
       <c r="D130" s="1"/>
       <c r="E130" s="1"/>
       <c r="F130" s="1"/>
       <c r="G130" s="1"/>
+      <c r="H130" s="1"/>
       <c r="I130" s="1" t="s">
-        <v>640</v>
+        <v>544</v>
       </c>
       <c r="J130" s="1"/>
       <c r="K130" s="1"/>
@@ -14460,7 +14447,7 @@
       <c r="O130" s="1"/>
       <c r="P130" s="1"/>
     </row>
-    <row r="131" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="131" spans="2:16" x14ac:dyDescent="0.3">
       <c r="B131" s="1" t="s">
         <v>10</v>
       </c>
@@ -14471,7 +14458,7 @@
         <v>634</v>
       </c>
       <c r="E131" s="1" t="s">
-        <v>744</v>
+        <v>740</v>
       </c>
       <c r="F131" s="1"/>
       <c r="G131" s="1"/>
@@ -14487,7 +14474,7 @@
       <c r="O131" s="1"/>
       <c r="P131" s="1"/>
     </row>
-    <row r="132" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="132" spans="2:16" x14ac:dyDescent="0.3">
       <c r="B132" s="1" t="s">
         <v>10</v>
       </c>
@@ -14498,7 +14485,7 @@
         <v>635</v>
       </c>
       <c r="E132" s="1" t="s">
-        <v>745</v>
+        <v>741</v>
       </c>
       <c r="F132" s="1"/>
       <c r="G132" s="1"/>
@@ -14514,7 +14501,7 @@
       <c r="O132" s="1"/>
       <c r="P132" s="1"/>
     </row>
-    <row r="133" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="133" spans="2:16" x14ac:dyDescent="0.3">
       <c r="B133" s="1" t="s">
         <v>10</v>
       </c>
@@ -14525,7 +14512,7 @@
         <v>636</v>
       </c>
       <c r="E133" s="1" t="s">
-        <v>746</v>
+        <v>742</v>
       </c>
       <c r="F133" s="1"/>
       <c r="G133" s="1"/>
@@ -14541,7 +14528,7 @@
       <c r="O133" s="1"/>
       <c r="P133" s="1"/>
     </row>
-    <row r="134" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="134" spans="2:16" x14ac:dyDescent="0.3">
       <c r="B134" s="1" t="s">
         <v>10</v>
       </c>
@@ -14549,10 +14536,10 @@
         <v>16</v>
       </c>
       <c r="D134" s="1" t="s">
-        <v>641</v>
+        <v>785</v>
       </c>
       <c r="E134" s="1" t="s">
-        <v>747</v>
+        <v>743</v>
       </c>
       <c r="F134" s="1"/>
       <c r="G134" s="1"/>
@@ -14567,7 +14554,7 @@
       <c r="O134" s="1"/>
       <c r="P134" s="1"/>
     </row>
-    <row r="135" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="135" spans="2:16" x14ac:dyDescent="0.3">
       <c r="B135" s="1" t="s">
         <v>546</v>
       </c>
@@ -14586,7 +14573,7 @@
       <c r="O135" s="1"/>
       <c r="P135" s="1"/>
     </row>
-    <row r="136" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="136" spans="2:16" x14ac:dyDescent="0.3">
       <c r="B136" s="1" t="s">
         <v>2</v>
       </c>
@@ -14609,7 +14596,7 @@
       </c>
       <c r="P136" s="1"/>
     </row>
-    <row r="137" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="137" spans="2:16" x14ac:dyDescent="0.3">
       <c r="B137" s="1" t="s">
         <v>59</v>
       </c>
@@ -14630,9 +14617,9 @@
         <v>545</v>
       </c>
     </row>
-    <row r="138" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="138" spans="2:16" x14ac:dyDescent="0.3">
       <c r="B138" s="1" t="s">
-        <v>783</v>
+        <v>779</v>
       </c>
       <c r="C138" s="1"/>
       <c r="D138" s="1"/>
@@ -14642,12 +14629,12 @@
       <c r="H138" s="1"/>
       <c r="I138" s="1"/>
       <c r="J138" s="1" t="s">
-        <v>785</v>
+        <v>781</v>
       </c>
       <c r="K138" s="1"/>
       <c r="L138" s="1"/>
       <c r="M138" s="1" t="s">
-        <v>787</v>
+        <v>783</v>
       </c>
       <c r="N138" s="1" t="s">
         <v>106</v>
@@ -14655,7 +14642,7 @@
       <c r="O138" s="1"/>
       <c r="P138" s="1"/>
     </row>
-    <row r="139" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="139" spans="2:16" x14ac:dyDescent="0.3">
       <c r="B139" s="1" t="s">
         <v>546</v>
       </c>
@@ -14676,18 +14663,18 @@
       <c r="O139" s="1"/>
       <c r="P139" s="1"/>
     </row>
-    <row r="140" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="140" spans="2:16" x14ac:dyDescent="0.3">
       <c r="B140" s="1" t="s">
         <v>10</v>
       </c>
       <c r="C140" s="1" t="s">
-        <v>670</v>
+        <v>666</v>
       </c>
       <c r="D140" s="1" t="s">
-        <v>642</v>
+        <v>638</v>
       </c>
       <c r="E140" s="1" t="s">
-        <v>748</v>
+        <v>744</v>
       </c>
       <c r="F140" s="1" t="s">
         <v>556</v>
@@ -14696,7 +14683,7 @@
         <v>12</v>
       </c>
       <c r="H140" s="1" t="s">
-        <v>643</v>
+        <v>639</v>
       </c>
       <c r="I140" s="1"/>
       <c r="J140" s="1"/>
@@ -14709,7 +14696,7 @@
       <c r="O140" s="1"/>
       <c r="P140" s="1"/>
     </row>
-    <row r="141" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="141" spans="2:16" x14ac:dyDescent="0.3">
       <c r="B141" s="1" t="s">
         <v>10</v>
       </c>
@@ -14717,10 +14704,10 @@
         <v>24</v>
       </c>
       <c r="D141" s="1" t="s">
-        <v>644</v>
+        <v>640</v>
       </c>
       <c r="E141" s="1" t="s">
-        <v>749</v>
+        <v>745</v>
       </c>
       <c r="F141" s="1" t="s">
         <v>557</v>
@@ -14729,7 +14716,7 @@
         <v>20</v>
       </c>
       <c r="H141" s="1" t="s">
-        <v>645</v>
+        <v>641</v>
       </c>
       <c r="I141" s="1"/>
       <c r="J141" s="1"/>
@@ -14742,7 +14729,7 @@
       <c r="O141" s="1"/>
       <c r="P141" s="1"/>
     </row>
-    <row r="142" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="142" spans="2:16" x14ac:dyDescent="0.3">
       <c r="B142" s="1" t="s">
         <v>10</v>
       </c>
@@ -14750,10 +14737,10 @@
         <v>16</v>
       </c>
       <c r="D142" s="1" t="s">
-        <v>646</v>
+        <v>642</v>
       </c>
       <c r="E142" s="1" t="s">
-        <v>750</v>
+        <v>746</v>
       </c>
       <c r="F142" s="1" t="s">
         <v>293</v>
@@ -14762,7 +14749,7 @@
         <v>5</v>
       </c>
       <c r="H142" t="s">
-        <v>647</v>
+        <v>643</v>
       </c>
       <c r="I142" s="1"/>
       <c r="J142" s="1"/>
@@ -14775,7 +14762,7 @@
       <c r="O142" s="1"/>
       <c r="P142" s="1"/>
     </row>
-    <row r="143" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="143" spans="2:16" x14ac:dyDescent="0.3">
       <c r="B143" s="1" t="s">
         <v>10</v>
       </c>
@@ -14783,10 +14770,10 @@
         <v>24</v>
       </c>
       <c r="D143" s="1" t="s">
-        <v>648</v>
+        <v>644</v>
       </c>
       <c r="E143" s="1" t="s">
-        <v>751</v>
+        <v>747</v>
       </c>
       <c r="F143" s="1" t="s">
         <v>557</v>
@@ -14808,7 +14795,7 @@
       <c r="O143" s="1"/>
       <c r="P143" s="1"/>
     </row>
-    <row r="144" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="144" spans="2:16" x14ac:dyDescent="0.3">
       <c r="B144" s="1" t="s">
         <v>10</v>
       </c>
@@ -14816,10 +14803,10 @@
         <v>24</v>
       </c>
       <c r="D144" s="1" t="s">
-        <v>649</v>
+        <v>645</v>
       </c>
       <c r="E144" s="1" t="s">
-        <v>752</v>
+        <v>748</v>
       </c>
       <c r="F144" s="1"/>
       <c r="G144" s="1"/>
@@ -14843,10 +14830,10 @@
         <v>16</v>
       </c>
       <c r="D145" s="1" t="s">
-        <v>650</v>
+        <v>646</v>
       </c>
       <c r="E145" s="1" t="s">
-        <v>753</v>
+        <v>749</v>
       </c>
       <c r="F145" s="1" t="s">
         <v>293</v>
@@ -14855,7 +14842,7 @@
         <v>5</v>
       </c>
       <c r="H145" t="s">
-        <v>781</v>
+        <v>777</v>
       </c>
       <c r="I145" s="1"/>
       <c r="J145" s="1"/>
@@ -14876,10 +14863,10 @@
         <v>16</v>
       </c>
       <c r="D146" s="1" t="s">
-        <v>651</v>
+        <v>647</v>
       </c>
       <c r="E146" s="1" t="s">
-        <v>754</v>
+        <v>750</v>
       </c>
       <c r="F146" s="1" t="s">
         <v>293</v>
@@ -14888,7 +14875,7 @@
         <v>5</v>
       </c>
       <c r="H146" t="s">
-        <v>652</v>
+        <v>648</v>
       </c>
       <c r="I146" s="1"/>
       <c r="J146" s="1"/>
@@ -14909,10 +14896,10 @@
         <v>91</v>
       </c>
       <c r="D147" s="1" t="s">
-        <v>653</v>
+        <v>649</v>
       </c>
       <c r="E147" s="1" t="s">
-        <v>755</v>
+        <v>751</v>
       </c>
       <c r="F147" s="1"/>
       <c r="G147" s="1"/>
@@ -14936,10 +14923,10 @@
         <v>9</v>
       </c>
       <c r="D148" s="1" t="s">
-        <v>654</v>
+        <v>650</v>
       </c>
       <c r="E148" s="1" t="s">
-        <v>756</v>
+        <v>752</v>
       </c>
       <c r="F148" s="1" t="s">
         <v>556</v>
@@ -14969,10 +14956,10 @@
         <v>9</v>
       </c>
       <c r="D149" s="1" t="s">
-        <v>655</v>
+        <v>651</v>
       </c>
       <c r="E149" s="1" t="s">
-        <v>757</v>
+        <v>753</v>
       </c>
       <c r="F149" s="1"/>
       <c r="G149" s="1"/>
@@ -14996,10 +14983,10 @@
         <v>16</v>
       </c>
       <c r="D150" s="1" t="s">
-        <v>656</v>
+        <v>652</v>
       </c>
       <c r="E150" s="1" t="s">
-        <v>758</v>
+        <v>754</v>
       </c>
       <c r="F150" s="1" t="s">
         <v>293</v>
@@ -15008,7 +14995,7 @@
         <v>5</v>
       </c>
       <c r="H150" t="s">
-        <v>657</v>
+        <v>653</v>
       </c>
       <c r="I150" s="1"/>
       <c r="J150" s="1"/>
@@ -15029,10 +15016,10 @@
         <v>9</v>
       </c>
       <c r="D151" s="1" t="s">
-        <v>658</v>
+        <v>654</v>
       </c>
       <c r="E151" s="1" t="s">
-        <v>759</v>
+        <v>755</v>
       </c>
       <c r="F151" s="1" t="s">
         <v>556</v>
@@ -15062,10 +15049,10 @@
         <v>9</v>
       </c>
       <c r="D152" s="1" t="s">
-        <v>659</v>
+        <v>655</v>
       </c>
       <c r="E152" s="1" t="s">
-        <v>760</v>
+        <v>756</v>
       </c>
       <c r="F152" s="1"/>
       <c r="G152" s="1"/>
@@ -15089,10 +15076,10 @@
         <v>9</v>
       </c>
       <c r="D153" s="1" t="s">
-        <v>660</v>
+        <v>656</v>
       </c>
       <c r="E153" s="1" t="s">
-        <v>761</v>
+        <v>757</v>
       </c>
       <c r="F153" s="1"/>
       <c r="G153" s="1"/>
@@ -15116,10 +15103,10 @@
         <v>91</v>
       </c>
       <c r="D154" s="1" t="s">
-        <v>661</v>
+        <v>657</v>
       </c>
       <c r="E154" s="1" t="s">
-        <v>762</v>
+        <v>758</v>
       </c>
       <c r="F154" s="1" t="s">
         <v>52</v>
@@ -15145,10 +15132,10 @@
         <v>16</v>
       </c>
       <c r="D155" s="1" t="s">
-        <v>662</v>
+        <v>658</v>
       </c>
       <c r="E155" s="1" t="s">
-        <v>763</v>
+        <v>759</v>
       </c>
       <c r="F155" s="1" t="s">
         <v>293</v>
@@ -15178,10 +15165,10 @@
         <v>91</v>
       </c>
       <c r="D156" s="1" t="s">
-        <v>663</v>
+        <v>659</v>
       </c>
       <c r="E156" s="1" t="s">
-        <v>764</v>
+        <v>760</v>
       </c>
       <c r="F156" s="1"/>
       <c r="G156" s="1"/>
@@ -15205,10 +15192,10 @@
         <v>16</v>
       </c>
       <c r="D157" s="1" t="s">
-        <v>664</v>
+        <v>660</v>
       </c>
       <c r="E157" s="1" t="s">
-        <v>765</v>
+        <v>761</v>
       </c>
       <c r="F157" s="1" t="s">
         <v>293</v>
@@ -15217,7 +15204,7 @@
         <v>20</v>
       </c>
       <c r="H157" t="s">
-        <v>665</v>
+        <v>661</v>
       </c>
       <c r="I157" s="1"/>
       <c r="J157" s="1"/>
@@ -15238,10 +15225,10 @@
         <v>91</v>
       </c>
       <c r="D158" s="1" t="s">
-        <v>666</v>
+        <v>662</v>
       </c>
       <c r="E158" s="1" t="s">
-        <v>766</v>
+        <v>762</v>
       </c>
       <c r="F158" s="1"/>
       <c r="G158" s="1"/>
@@ -15349,10 +15336,10 @@
         <v>24</v>
       </c>
       <c r="D163" s="1" t="s">
-        <v>667</v>
+        <v>663</v>
       </c>
       <c r="E163" s="1" t="s">
-        <v>767</v>
+        <v>763</v>
       </c>
       <c r="F163" s="1" t="s">
         <v>557</v>
@@ -15361,7 +15348,7 @@
         <v>12</v>
       </c>
       <c r="H163" s="1" t="s">
-        <v>782</v>
+        <v>778</v>
       </c>
       <c r="I163" s="1"/>
       <c r="J163" s="1"/>
@@ -15382,10 +15369,10 @@
         <v>9</v>
       </c>
       <c r="D164" s="1" t="s">
-        <v>668</v>
+        <v>664</v>
       </c>
       <c r="E164" s="1" t="s">
-        <v>768</v>
+        <v>764</v>
       </c>
       <c r="F164" s="1" t="s">
         <v>556</v>
@@ -15394,7 +15381,7 @@
         <v>5</v>
       </c>
       <c r="H164" s="1" t="s">
-        <v>669</v>
+        <v>665</v>
       </c>
       <c r="I164" s="1"/>
       <c r="J164" s="1"/>

</xml_diff>